<commit_message>
feat(guidance): GCForm-03 Excel-file preview with value-only template fill, centered dates, ADM consult reviewer routing
</commit_message>
<xml_diff>
--- a/frontend/public/referral forms/Referral Form - GCForm-03 v11.xlsx
+++ b/frontend/public/referral forms/Referral Form - GCForm-03 v11.xlsx
@@ -161,7 +161,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -182,6 +182,13 @@
       <b/>
       <color rgb="FF0B2C6F"/>
       <sz val="18"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="12"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -364,7 +371,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -375,11 +382,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -406,10 +413,16 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -420,8 +433,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
   </cellXfs>
@@ -1094,7 +1110,7 @@
       <c r="E20" s="18"/>
       <c r="F20" s="18"/>
       <c r="G20" s="18"/>
-      <c r="H20" s="18"/>
+      <c r="H20" s="19"/>
       <c r="I20" s="18"/>
       <c r="J20" s="18"/>
     </row>
@@ -1108,7 +1124,7 @@
       <c r="E21" s="18"/>
       <c r="F21" s="18"/>
       <c r="G21" s="18"/>
-      <c r="H21" s="18"/>
+      <c r="H21" s="19"/>
       <c r="I21" s="18"/>
       <c r="J21" s="18"/>
     </row>
@@ -1122,7 +1138,7 @@
       <c r="E22" s="18"/>
       <c r="F22" s="18"/>
       <c r="G22" s="18"/>
-      <c r="H22" s="18"/>
+      <c r="H22" s="19"/>
       <c r="I22" s="18"/>
       <c r="J22" s="18"/>
     </row>
@@ -1136,7 +1152,7 @@
       <c r="E23" s="18"/>
       <c r="F23" s="18"/>
       <c r="G23" s="18"/>
-      <c r="H23" s="18"/>
+      <c r="H23" s="19"/>
       <c r="I23" s="18"/>
       <c r="J23" s="18"/>
     </row>
@@ -1150,7 +1166,7 @@
       <c r="E24" s="18"/>
       <c r="F24" s="18"/>
       <c r="G24" s="18"/>
-      <c r="H24" s="18"/>
+      <c r="H24" s="19"/>
       <c r="I24" s="18"/>
       <c r="J24" s="18"/>
     </row>
@@ -1215,20 +1231,20 @@
       <c r="J29" s="1"/>
     </row>
     <row r="30" ht="20" customHeight="1" spans="6:10" x14ac:dyDescent="0.25">
-      <c r="F30" s="19" t="s">
+      <c r="F30" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="G30" s="19"/>
-      <c r="H30" s="19"/>
-      <c r="I30" s="19"/>
-      <c r="J30" s="19"/>
+      <c r="G30" s="20"/>
+      <c r="H30" s="20"/>
+      <c r="I30" s="20"/>
+      <c r="J30" s="20"/>
     </row>
     <row r="31" ht="28" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
         <v>31</v>
       </c>
       <c r="B31" s="7"/>
-      <c r="C31" s="4" t="s">
+      <c r="C31" s="21" t="s">
         <v>11</v>
       </c>
       <c r="D31" s="4"/>
@@ -1236,7 +1252,7 @@
       <c r="F31" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="G31" s="4" t="s">
+      <c r="G31" s="21" t="s">
         <v>11</v>
       </c>
       <c r="H31" s="4"/>
@@ -1244,25 +1260,25 @@
       <c r="J31" s="4"/>
     </row>
     <row r="32" ht="20" customHeight="1" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C32" s="19" t="s">
+      <c r="C32" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="D32" s="19"/>
-      <c r="E32" s="19"/>
+      <c r="D32" s="20"/>
+      <c r="E32" s="20"/>
     </row>
     <row r="33" ht="14" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A33" s="20" t="s">
+      <c r="A33" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
-      <c r="D33" s="20"/>
-      <c r="E33" s="20"/>
-      <c r="F33" s="20"/>
-      <c r="G33" s="20"/>
-      <c r="H33" s="20"/>
-      <c r="I33" s="20"/>
-      <c r="J33" s="20"/>
+      <c r="B33" s="22"/>
+      <c r="C33" s="22"/>
+      <c r="D33" s="22"/>
+      <c r="E33" s="22"/>
+      <c r="F33" s="22"/>
+      <c r="G33" s="22"/>
+      <c r="H33" s="22"/>
+      <c r="I33" s="22"/>
+      <c r="J33" s="22"/>
     </row>
     <row r="34" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
@@ -1279,74 +1295,74 @@
       <c r="J34" s="2"/>
     </row>
     <row r="35" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A35" s="21" t="s">
+      <c r="A35" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="B35" s="22"/>
+      <c r="B35" s="24"/>
       <c r="C35" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="D35" s="21" t="s">
+      <c r="D35" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="E35" s="22"/>
-      <c r="F35" s="21" t="s">
+      <c r="E35" s="24"/>
+      <c r="F35" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="G35" s="22"/>
-      <c r="H35" s="21" t="s">
+      <c r="G35" s="24"/>
+      <c r="H35" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="I35" s="23"/>
-      <c r="J35" s="22"/>
+      <c r="I35" s="25"/>
+      <c r="J35" s="24"/>
     </row>
     <row r="36" ht="28" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" s="24" t="s">
+      <c r="A36" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="B36" s="22"/>
-      <c r="C36" s="25" t="s">
+      <c r="B36" s="24"/>
+      <c r="C36" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="D36" s="26"/>
-      <c r="E36" s="22"/>
-      <c r="F36" s="26"/>
-      <c r="G36" s="22"/>
-      <c r="H36" s="26"/>
-      <c r="I36" s="23"/>
-      <c r="J36" s="22"/>
+      <c r="D36" s="28"/>
+      <c r="E36" s="24"/>
+      <c r="F36" s="29"/>
+      <c r="G36" s="24"/>
+      <c r="H36" s="29"/>
+      <c r="I36" s="25"/>
+      <c r="J36" s="24"/>
     </row>
     <row r="37" ht="28" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A37" s="24" t="s">
+      <c r="A37" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="B37" s="22"/>
-      <c r="C37" s="25" t="s">
+      <c r="B37" s="24"/>
+      <c r="C37" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="D37" s="26"/>
-      <c r="E37" s="22"/>
-      <c r="F37" s="26"/>
-      <c r="G37" s="22"/>
-      <c r="H37" s="26"/>
-      <c r="I37" s="23"/>
-      <c r="J37" s="22"/>
+      <c r="D37" s="28"/>
+      <c r="E37" s="24"/>
+      <c r="F37" s="29"/>
+      <c r="G37" s="24"/>
+      <c r="H37" s="29"/>
+      <c r="I37" s="25"/>
+      <c r="J37" s="24"/>
     </row>
     <row r="38" ht="28" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A38" s="24" t="s">
+      <c r="A38" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="B38" s="22"/>
-      <c r="C38" s="25" t="s">
+      <c r="B38" s="24"/>
+      <c r="C38" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="D38" s="26"/>
-      <c r="E38" s="22"/>
-      <c r="F38" s="26"/>
-      <c r="G38" s="22"/>
-      <c r="H38" s="26"/>
-      <c r="I38" s="23"/>
-      <c r="J38" s="22"/>
+      <c r="D38" s="28"/>
+      <c r="E38" s="24"/>
+      <c r="F38" s="29"/>
+      <c r="G38" s="24"/>
+      <c r="H38" s="29"/>
+      <c r="I38" s="25"/>
+      <c r="J38" s="24"/>
     </row>
     <row r="39" ht="28" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
@@ -1445,7 +1461,7 @@
       <c r="C46" s="4"/>
       <c r="D46" s="4"/>
       <c r="E46" s="4"/>
-      <c r="G46" s="4" t="s">
+      <c r="G46" s="21" t="s">
         <v>11</v>
       </c>
       <c r="H46" s="4"/>
@@ -1468,18 +1484,18 @@
       <c r="J47" s="1"/>
     </row>
     <row r="48" ht="14" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A48" s="20" t="s">
+      <c r="A48" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="B48" s="20"/>
-      <c r="C48" s="20"/>
-      <c r="D48" s="20"/>
-      <c r="E48" s="20"/>
-      <c r="F48" s="20"/>
-      <c r="G48" s="20"/>
-      <c r="H48" s="20"/>
-      <c r="I48" s="20"/>
-      <c r="J48" s="20"/>
+      <c r="B48" s="22"/>
+      <c r="C48" s="22"/>
+      <c r="D48" s="22"/>
+      <c r="E48" s="22"/>
+      <c r="F48" s="22"/>
+      <c r="G48" s="22"/>
+      <c r="H48" s="22"/>
+      <c r="I48" s="22"/>
+      <c r="J48" s="22"/>
     </row>
     <row r="49" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="17" t="s">
@@ -1502,16 +1518,16 @@
       <c r="J49" s="17"/>
     </row>
     <row r="50" ht="24" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A50" s="26"/>
-      <c r="B50" s="22"/>
-      <c r="C50" s="26"/>
-      <c r="D50" s="23"/>
-      <c r="E50" s="22"/>
-      <c r="F50" s="26"/>
-      <c r="G50" s="22"/>
-      <c r="H50" s="26"/>
-      <c r="I50" s="23"/>
-      <c r="J50" s="22"/>
+      <c r="A50" s="29"/>
+      <c r="B50" s="24"/>
+      <c r="C50" s="29"/>
+      <c r="D50" s="25"/>
+      <c r="E50" s="24"/>
+      <c r="F50" s="29"/>
+      <c r="G50" s="24"/>
+      <c r="H50" s="29"/>
+      <c r="I50" s="25"/>
+      <c r="J50" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="66">
@@ -1584,7 +1600,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <headerFooter>
     <oddFooter>&amp;CPage &amp;P of &amp;N</oddFooter>
   </headerFooter>

</xml_diff>